<commit_message>
D3 in BOM updated
</commit_message>
<xml_diff>
--- a/Design-Files/Interface-Board-v4.0/BOM/Client-BOM-Interface-Board-v4.0.xlsx
+++ b/Design-Files/Interface-Board-v4.0/BOM/Client-BOM-Interface-Board-v4.0.xlsx
@@ -1,20 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ChristianRaun-EthercatDesign\Design-Files\Interface-Board-v4.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A52DFA-068A-4788-B037-F81A3457BCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -282,9 +297,6 @@
     <t>TVS DIODE 48VWM 77.4VC DO214AC</t>
   </si>
   <si>
-    <t>Schottky Barrier Diode SK36, DO-214AB, 3A/60V</t>
-  </si>
-  <si>
     <t>TVS DIODE 3.3VWM 11.5VC MICROSMP</t>
   </si>
   <si>
@@ -757,12 +769,15 @@
   </si>
   <si>
     <t>CC0201KRX5R8BB223</t>
+  </si>
+  <si>
+    <t>60V Independent 700mV@3A 3A SMA(DO-214AC) Schottky Diodes ROHS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -976,9 +991,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -987,6 +999,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1273,27 +1288,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.44140625" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1302,11 +1317,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1321,25 +1336,25 @@
         <v>66</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1355,23 +1370,23 @@
         <v>67</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B50" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1387,23 +1402,23 @@
         <v>68</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1419,23 +1434,23 @@
         <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1451,23 +1466,23 @@
         <v>70</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1483,23 +1498,23 @@
         <v>71</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1515,23 +1530,23 @@
         <v>72</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1547,23 +1562,23 @@
         <v>73</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1579,23 +1594,23 @@
         <v>74</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J10" s="9">
         <v>2</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1611,23 +1626,23 @@
         <v>75</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1643,23 +1658,23 @@
         <v>76</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J12" s="9">
         <v>3</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1675,23 +1690,23 @@
         <v>77</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1707,23 +1722,23 @@
         <v>78</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J14" s="9">
         <v>2</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1739,23 +1754,23 @@
         <v>79</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J15" s="7">
         <v>4</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1771,23 +1786,23 @@
         <v>80</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1803,23 +1818,23 @@
         <v>81</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="J17" s="7">
         <v>4</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1835,23 +1850,23 @@
         <v>82</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J18" s="9">
         <v>8</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1867,23 +1882,23 @@
         <v>83</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="J19" s="7">
         <v>2</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1899,23 +1914,23 @@
         <v>84</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1931,23 +1946,23 @@
         <v>85</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1963,23 +1978,23 @@
         <v>86</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1992,26 +2007,26 @@
         <v>37</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>87</v>
+        <v>245</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -2024,26 +2039,26 @@
         <v>38</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -2056,26 +2071,26 @@
         <v>39</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -2088,26 +2103,26 @@
         <v>40</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -2120,26 +2135,26 @@
         <v>41</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J27" s="7">
         <v>2</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -2152,26 +2167,26 @@
         <v>42</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J28" s="9">
         <v>2</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -2184,26 +2199,26 @@
         <v>43</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2216,26 +2231,26 @@
         <v>44</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2248,26 +2263,26 @@
         <v>45</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2280,26 +2295,26 @@
         <v>46</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2312,26 +2327,26 @@
         <v>47</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2340,32 +2355,32 @@
       <c r="C34" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="F34" s="15" t="s">
+      <c r="E34" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="H34" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="G34" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="H34" s="15" t="s">
-        <v>241</v>
-      </c>
-      <c r="I34" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="J34" s="15">
+      <c r="I34" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="J34" s="14">
         <v>3</v>
       </c>
-      <c r="K34" s="17" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K34" s="16" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2378,26 +2393,26 @@
         <v>49</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2410,26 +2425,26 @@
         <v>50</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -2442,26 +2457,26 @@
         <v>51</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
       </c>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -2474,26 +2489,26 @@
         <v>52</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -2506,26 +2521,26 @@
         <v>53</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J39" s="7">
         <v>2</v>
       </c>
       <c r="K39" s="7"/>
     </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f t="shared" si="0"/>
@@ -2538,26 +2553,26 @@
         <v>54</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -2570,26 +2585,26 @@
         <v>55</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J41" s="7">
         <v>8</v>
       </c>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f t="shared" si="0"/>
@@ -2602,26 +2617,26 @@
         <v>56</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J42" s="9">
         <v>4</v>
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
@@ -2634,26 +2649,26 @@
         <v>57</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J43" s="7">
         <v>2</v>
       </c>
       <c r="K43" s="7"/>
     </row>
-    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -2666,26 +2681,26 @@
         <v>58</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J44" s="9">
         <v>8</v>
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
@@ -2698,26 +2713,26 @@
         <v>59</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
       </c>
       <c r="K45" s="7"/>
     </row>
-    <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
@@ -2730,26 +2745,26 @@
         <v>60</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
       </c>
       <c r="K46" s="9"/>
     </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
@@ -2762,26 +2777,26 @@
         <v>61</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -2794,26 +2809,26 @@
         <v>62</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
       </c>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
@@ -2826,26 +2841,26 @@
         <v>63</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
       </c>
       <c r="K49" s="7"/>
     </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
@@ -2858,26 +2873,26 @@
         <v>64</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
       <c r="K50" s="9"/>
     </row>
-    <row r="51" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
@@ -2890,19 +2905,19 @@
         <v>65</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J51" s="7">
         <v>4</v>

</xml_diff>